<commit_message>
تعديل يدوي في شيت Card1 by admin at 2026-09-21 10:48:00
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -19912,15 +19912,31 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1473</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>20/9/2026</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card19 by admin at 2026-09-21 10:50:13
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -27539,15 +27539,31 @@
           <t>1500</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1459</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>16/9/2026</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card21 by admin at 2026-09-21 10:52:30
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -24184,15 +24184,31 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1423</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>15/9/2026</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>

</xml_diff>

<commit_message>
تعديل يدوي في شيت Card20 by admin at 2026-09-21 10:54:45
</commit_message>
<xml_diff>
--- a/l4.xlsx
+++ b/l4.xlsx
@@ -25864,15 +25864,31 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1447</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>13/9/2026</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>

</xml_diff>